<commit_message>
Audit monthly components and full market coverage matrix
</commit_message>
<xml_diff>
--- a/market-history/research/regime190/inventory_190.xlsx
+++ b/market-history/research/regime190/inventory_190.xlsx
@@ -11309,13 +11309,21 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>0</v>
-      </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -11323,13 +11331,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
-      <c r="O117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>710d74c96cd37e3eb709648ea5f9321d9b6c268224c6fdf925e8c800ebbad776</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="P117" t="n">
-        <v>0</v>
+        <v>202</v>
       </c>
       <c r="Q117" t="n">
         <v>0</v>
@@ -11338,32 +11366,32 @@
       <c r="S117" t="inlineStr"/>
       <c r="T117" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V117" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; US 2Y missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y117" t="inlineStr">
         <is>
-          <t>FRED/ALFRED·OFR·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -12139,13 +12167,21 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>0</v>
-      </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>market-history/data/korea-market-monthly.csv</t>
+        </is>
+      </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -12153,13 +12189,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
-      <c r="M127" t="inlineStr"/>
-      <c r="N127" t="inlineStr"/>
-      <c r="O127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>market-history/data/korea-market-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>d54563e43e5d043d8eca400c21d95256cce57ee2138eef1eb2f38f87f8d5a20a</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="P127" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="Q127" t="n">
         <v>0</v>
@@ -12168,32 +12224,32 @@
       <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; daily FX history and close time missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
         <is>
-          <t>거래소·FRED·공식통계·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -12305,13 +12361,21 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>0</v>
-      </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -12319,13 +12383,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
-      <c r="N129" t="inlineStr"/>
-      <c r="O129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>710d74c96cd37e3eb709648ea5f9321d9b6c268224c6fdf925e8c800ebbad776</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="P129" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="Q129" t="n">
         <v>0</v>
@@ -12334,32 +12418,32 @@
       <c r="S129" t="inlineStr"/>
       <c r="T129" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V129" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; yuan and direct yen series missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
         <is>
-          <t>거래소·FRED·공식통계·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -12554,13 +12638,21 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>0</v>
-      </c>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>market-history/data/us-stock-market-monthly.csv</t>
+        </is>
+      </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -12568,13 +12660,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr"/>
-      <c r="N132" t="inlineStr"/>
-      <c r="O132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>market-history/data/us-stock-market-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>74f0e755b749faae6e0d028f5d1c6f600572494cfd286c072dd7b880eb1fb27d</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="P132" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="Q132" t="n">
         <v>0</v>
@@ -12583,32 +12695,32 @@
       <c r="S132" t="inlineStr"/>
       <c r="T132" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V132" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; NASDAQ and SOX missing; price identity unverified; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y132" t="inlineStr">
         <is>
-          <t>거래소·FRED·공식통계·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -12803,13 +12915,21 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>0</v>
-      </c>
-      <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-commodities-monthly.csv</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -12817,13 +12937,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-commodities-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>4675274c132fc62254a9fc744113517f5f987215b68ccc5f5556d875b090489a</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="P135" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="Q135" t="n">
         <v>0</v>
@@ -12832,32 +12972,32 @@
       <c r="S135" t="inlineStr"/>
       <c r="T135" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V135" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; natural gas missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y135" t="inlineStr">
         <is>
-          <t>거래소·FRED·공식통계·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -12886,13 +13026,21 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>0</v>
-      </c>
-      <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-commodities-monthly.csv</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -12900,13 +13048,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-commodities-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>4675274c132fc62254a9fc744113517f5f987215b68ccc5f5556d875b090489a</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="P136" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="Q136" t="n">
         <v>0</v>
@@ -12915,32 +13083,32 @@
       <c r="S136" t="inlineStr"/>
       <c r="T136" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V136" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; silver, copper, iron ore missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y136" t="inlineStr">
         <is>
-          <t>거래소·FRED·공식통계·시장 공급사</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>
@@ -13550,13 +13718,21 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>0</v>
-      </c>
-      <c r="G144" t="inlineStr"/>
-      <c r="H144" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>existing monthly repository CSV</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>upstream_license_unverified</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -13564,13 +13740,33 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
-      <c r="O144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>market-history/data/macro-cpi-rates-monthly.csv</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>710d74c96cd37e3eb709648ea5f9321d9b6c268224c6fdf925e8c800ebbad776</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="P144" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="Q144" t="n">
         <v>0</v>
@@ -13579,32 +13775,32 @@
       <c r="S144" t="inlineStr"/>
       <c r="T144" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U144" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V144" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Monthly component only; core CPI missing; publication time and vintage unavailable</t>
         </is>
       </c>
       <c r="X144" t="inlineStr">
         <is>
-          <t>Try official source, then licensed alternative, with bounded requests</t>
+          <t>Collect missing components and first-release vintages</t>
         </is>
       </c>
       <c r="Y144" t="inlineStr">
         <is>
-          <t>한국은행 ECOS·KOSIS·관세청·FRED</t>
+          <t>Only listed monthly components observed; complete indicator valid_count=0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record bounded source probes and add safe metadata publisher
</commit_message>
<xml_diff>
--- a/market-history/research/regime190/inventory_190.xlsx
+++ b/market-history/research/regime190/inventory_190.xlsx
@@ -12287,7 +12287,7 @@
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U78" t="inlineStr">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X78" t="inlineStr">
@@ -12319,29 +12319,29 @@
         <v>1</v>
       </c>
       <c r="AA78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB78" t="n">
         <v>0</v>
       </c>
       <c r="AC78" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.102915+00:00</t>
+          <t>2026-10-27T15:49:57.888963+00:00</t>
         </is>
       </c>
       <c r="AD78" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "krx_microstructure", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE78" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF78" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG78" t="inlineStr">
@@ -12577,7 +12577,7 @@
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U80" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X80" t="inlineStr">
@@ -12609,29 +12609,29 @@
         <v>1</v>
       </c>
       <c r="AA80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB80" t="n">
         <v>0</v>
       </c>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.113613+00:00</t>
+          <t>2026-10-27T15:49:57.888963+00:00</t>
         </is>
       </c>
       <c r="AD80" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "krx_microstructure", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE80" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF80" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG80" t="inlineStr">
@@ -12708,7 +12708,7 @@
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U81" t="inlineStr">
@@ -12723,7 +12723,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
@@ -12740,29 +12740,29 @@
         <v>1</v>
       </c>
       <c r="AA81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB81" t="n">
         <v>0</v>
       </c>
       <c r="AC81" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.286328+00:00</t>
+          <t>2026-10-27T15:49:57.888963+00:00</t>
         </is>
       </c>
       <c r="AD81" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "krx_microstructure", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE81" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF81" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG81" t="inlineStr">
@@ -12839,7 +12839,7 @@
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U82" t="inlineStr">
@@ -12854,7 +12854,7 @@
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X82" t="inlineStr">
@@ -12871,29 +12871,29 @@
         <v>1</v>
       </c>
       <c r="AA82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB82" t="n">
         <v>0</v>
       </c>
       <c r="AC82" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.117197+00:00</t>
+          <t>2026-10-27T15:49:57.888963+00:00</t>
         </is>
       </c>
       <c r="AD82" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "krx_microstructure", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE82" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF82" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG82" t="inlineStr">
@@ -18565,7 +18565,7 @@
       <c r="S124" t="inlineStr"/>
       <c r="T124" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U124" t="inlineStr">
@@ -18580,7 +18580,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X124" t="inlineStr">
@@ -18597,29 +18597,29 @@
         <v>1</v>
       </c>
       <c r="AA124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB124" t="n">
         <v>0</v>
       </c>
       <c r="AC124" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:08.309101+00:00</t>
+          <t>2026-10-27T15:50:22.978147+00:00</t>
         </is>
       </c>
       <c r="AD124" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "fred_move_search", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE124" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF124" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG124" t="inlineStr">
@@ -18696,7 +18696,7 @@
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U125" t="inlineStr">
@@ -18711,7 +18711,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X125" t="inlineStr">
@@ -18728,29 +18728,29 @@
         <v>1</v>
       </c>
       <c r="AA125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB125" t="n">
         <v>0</v>
       </c>
       <c r="AC125" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:08.313438+00:00</t>
+          <t>2026-10-27T15:50:24.511897+00:00</t>
         </is>
       </c>
       <c r="AD125" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "fred_cds_search", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE125" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF125" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG125" t="inlineStr">
@@ -24297,8 +24297,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>https://www.bok.or.kr/portal/main/contents.do?menuNo=200755</t>
+        </is>
+      </c>
       <c r="I165" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24309,9 +24317,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>private:probe_bok_policy.html</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>fde19e52c9c6b42a7a37ee3938a6b587c4ade60d79ab836cb76f959115c20c7c</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N165" t="inlineStr"/>
       <c r="O165" t="inlineStr"/>
       <c r="P165" t="inlineStr">
@@ -24328,22 +24348,22 @@
       <c r="S165" t="inlineStr"/>
       <c r="T165" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U165" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V165" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W165" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X165" t="inlineStr">
@@ -24360,34 +24380,34 @@
         <v>1</v>
       </c>
       <c r="AA165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB165" t="n">
         <v>0</v>
       </c>
       <c r="AC165" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.542744+00:00</t>
+          <t>2026-10-27T15:50:01.674023+00:00</t>
         </is>
       </c>
       <c r="AD165" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "bok_policy", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE165" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF165" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG165" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH165" t="inlineStr">
@@ -24428,8 +24448,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/monetarypolicy/fomccalendars.htm</t>
+        </is>
+      </c>
       <c r="I166" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24440,9 +24468,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
-      <c r="M166" t="inlineStr"/>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>private:probe_fed_fomc.html</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>ddbc500359cb4f9c78b903eca20459e60b6f9c13be8b947b758b9d6d46393cdb</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N166" t="inlineStr"/>
       <c r="O166" t="inlineStr"/>
       <c r="P166" t="inlineStr">
@@ -24459,22 +24499,22 @@
       <c r="S166" t="inlineStr"/>
       <c r="T166" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U166" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V166" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W166" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X166" t="inlineStr">
@@ -24491,34 +24531,34 @@
         <v>1</v>
       </c>
       <c r="AA166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB166" t="n">
         <v>0</v>
       </c>
       <c r="AC166" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.548021+00:00</t>
+          <t>2026-10-27T15:50:03.107709+00:00</t>
         </is>
       </c>
       <c r="AD166" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "fed_fomc", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE166" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF166" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG166" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH166" t="inlineStr">
@@ -24559,8 +24599,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>https://www.treasurydirect.gov/auctions/announcements-data-results/</t>
+        </is>
+      </c>
       <c r="I167" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24571,9 +24619,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
-      <c r="M167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>private:probe_treasury_auction.html</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>830f98996908f6a9dcbe336552e405f7578c09a7024ced0c161730bcdcf99f6b</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="inlineStr"/>
       <c r="P167" t="inlineStr">
@@ -24590,22 +24650,22 @@
       <c r="S167" t="inlineStr"/>
       <c r="T167" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U167" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V167" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W167" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X167" t="inlineStr">
@@ -24622,34 +24682,34 @@
         <v>1</v>
       </c>
       <c r="AA167" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB167" t="n">
         <v>0</v>
       </c>
       <c r="AC167" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.090434+00:00</t>
+          <t>2026-10-27T15:50:04.406343+00:00</t>
         </is>
       </c>
       <c r="AD167" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "treasury_auction", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE167" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF167" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG167" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH167" t="inlineStr">
@@ -24690,8 +24750,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>https://app2.msci.com/webapp/index_ann/Announcement?doc_type=ANNOUNCEMENT&amp;format=html&amp;lang=en&amp;prod_type=STANDARD&amp;visibility=public</t>
+        </is>
+      </c>
       <c r="I168" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24702,9 +24770,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>private:probe_msci_review.html</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>e3f7caf9f0de25fcba472b537284fe25ce0bcb31377c97a373c03b158aa8da84</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr"/>
       <c r="P168" t="inlineStr">
@@ -24721,22 +24801,22 @@
       <c r="S168" t="inlineStr"/>
       <c r="T168" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U168" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V168" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W168" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X168" t="inlineStr">
@@ -24753,34 +24833,34 @@
         <v>1</v>
       </c>
       <c r="AA168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB168" t="n">
         <v>0</v>
       </c>
       <c r="AC168" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.551515+00:00</t>
+          <t>2026-10-27T15:50:07.147890+00:00</t>
         </is>
       </c>
       <c r="AD168" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "msci_review", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE168" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF168" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG168" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH168" t="inlineStr">
@@ -24821,8 +24901,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>https://www.fsc.go.kr/no010101</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24833,9 +24921,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>private:probe_fsc_policy.html</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>0747ab6927121b7b045c2958548a9d58d77d7989037d23465c2328ec0c934f5b</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N169" t="inlineStr"/>
       <c r="O169" t="inlineStr"/>
       <c r="P169" t="inlineStr">
@@ -24852,22 +24952,22 @@
       <c r="S169" t="inlineStr"/>
       <c r="T169" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V169" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W169" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X169" t="inlineStr">
@@ -24884,34 +24984,34 @@
         <v>1</v>
       </c>
       <c r="AA169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB169" t="n">
         <v>0</v>
       </c>
       <c r="AC169" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.556591+00:00</t>
+          <t>2026-10-27T15:50:08.585167+00:00</t>
         </is>
       </c>
       <c r="AD169" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "fsc_policy", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE169" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF169" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG169" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH169" t="inlineStr">
@@ -24952,8 +25052,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>https://www.ustr.gov/about-us/policy-offices/press-office/press-releases</t>
+        </is>
+      </c>
       <c r="I170" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -24964,9 +25072,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>private:probe_ustr_press.html</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>db2036f2d3a13e5c222dcb76015d38949796ebee113ffefd19924440802da197</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N170" t="inlineStr"/>
       <c r="O170" t="inlineStr"/>
       <c r="P170" t="inlineStr">
@@ -24983,22 +25103,22 @@
       <c r="S170" t="inlineStr"/>
       <c r="T170" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V170" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W170" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X170" t="inlineStr">
@@ -25015,34 +25135,34 @@
         <v>1</v>
       </c>
       <c r="AA170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB170" t="n">
         <v>0</v>
       </c>
       <c r="AC170" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.567897+00:00</t>
+          <t>2026-10-27T15:50:10.147024+00:00</t>
         </is>
       </c>
       <c r="AD170" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "ustr_press", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE170" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF170" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG170" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH170" t="inlineStr">
@@ -25083,8 +25203,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>https://www.boj.or.jp/en/mopo/mpmdeci/index.htm</t>
+        </is>
+      </c>
       <c r="I171" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -25095,9 +25223,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr"/>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>private:probe_boj_policy.html</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>a7abf675ec8d2c723c7e21de86ed7156e853f6a953caff170ebdbfc7f6d61c3b</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N171" t="inlineStr"/>
       <c r="O171" t="inlineStr"/>
       <c r="P171" t="inlineStr">
@@ -25114,22 +25254,22 @@
       <c r="S171" t="inlineStr"/>
       <c r="T171" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U171" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V171" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W171" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X171" t="inlineStr">
@@ -25146,34 +25286,34 @@
         <v>1</v>
       </c>
       <c r="AA171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB171" t="n">
         <v>0</v>
       </c>
       <c r="AC171" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:58.575177+00:00</t>
+          <t>2026-10-27T15:50:11.789693+00:00</t>
         </is>
       </c>
       <c r="AD171" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "boj_policy", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE171" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF171" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG171" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH171" t="inlineStr">
@@ -25214,8 +25354,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>official release archive page</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>https://ofac.treasury.gov/press-releases</t>
+        </is>
+      </c>
       <c r="I172" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -25226,9 +25374,21 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>private:probe_ofac_actions.html</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>11aa134ac2327ac058e4cccaedcf1a7e6c6e2e96ae993c78f2fb62264326b937</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>event_archive_unparsed</t>
+        </is>
+      </c>
       <c r="N172" t="inlineStr"/>
       <c r="O172" t="inlineStr"/>
       <c r="P172" t="inlineStr">
@@ -25245,22 +25405,22 @@
       <c r="S172" t="inlineStr"/>
       <c r="T172" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>원천 확보·계산 미완료</t>
         </is>
       </c>
       <c r="U172" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V172" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>UNPARSED_ARCHIVE</t>
         </is>
       </c>
       <c r="W172" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Official page downloaded and hashed, but indicator-specific historical events and publication times are unparsed</t>
         </is>
       </c>
       <c r="X172" t="inlineStr">
@@ -25277,34 +25437,34 @@
         <v>1</v>
       </c>
       <c r="AA172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB172" t="n">
         <v>0</v>
       </c>
       <c r="AC172" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.093358+00:00</t>
+          <t>2026-10-27T15:50:13.750881+00:00</t>
         </is>
       </c>
       <c r="AD172" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "ofac_actions", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE172" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Official release archive page saved, but historical event rows and publication times not yet extracted</t>
         </is>
       </c>
       <c r="AF172" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Parse dated archive releases, filter indicator events, and verify release time</t>
         </is>
       </c>
       <c r="AG172" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH172" t="inlineStr">
@@ -25376,7 +25536,7 @@
       <c r="S173" t="inlineStr"/>
       <c r="T173" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U173" t="inlineStr">
@@ -25391,7 +25551,7 @@
       </c>
       <c r="W173" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X173" t="inlineStr">
@@ -25408,29 +25568,29 @@
         <v>1</v>
       </c>
       <c r="AA173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB173" t="n">
         <v>0</v>
       </c>
       <c r="AC173" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.098110+00:00</t>
+          <t>2026-10-27T15:50:16.238141+00:00</t>
         </is>
       </c>
       <c r="AD173" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "krx_options_rules", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE173" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF173" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG173" t="inlineStr">
@@ -25507,7 +25667,7 @@
       <c r="S174" t="inlineStr"/>
       <c r="T174" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U174" t="inlineStr">
@@ -25522,7 +25682,7 @@
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X174" t="inlineStr">
@@ -25539,29 +25699,29 @@
         <v>1</v>
       </c>
       <c r="AA174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB174" t="n">
         <v>0</v>
       </c>
       <c r="AC174" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.103803+00:00</t>
+          <t>2026-10-27T15:50:25.925562+00:00</t>
         </is>
       </c>
       <c r="AD174" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "dart_filings_candidate", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE174" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF174" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG174" t="inlineStr">
@@ -25956,7 +26116,7 @@
       <c r="S177" t="inlineStr"/>
       <c r="T177" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U177" t="inlineStr">
@@ -25971,7 +26131,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X177" t="inlineStr">
@@ -25991,26 +26151,26 @@
         <v>0</v>
       </c>
       <c r="AB177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC177" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.111190+00:00</t>
+          <t>2026-10-27T15:50:27.104971+00:00</t>
         </is>
       </c>
       <c r="AD177" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "local_youtube_report", "http_status": null, "result": "DERIVED_REPORTS_ONLY_NO_TRANSCRIPT_OR_CHART_TIME"}</t>
         </is>
       </c>
       <c r="AE177" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF177" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG177" t="inlineStr">
@@ -26087,7 +26247,7 @@
       <c r="S178" t="inlineStr"/>
       <c r="T178" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U178" t="inlineStr">
@@ -26102,7 +26262,7 @@
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X178" t="inlineStr">
@@ -26119,29 +26279,29 @@
         <v>1</v>
       </c>
       <c r="AA178" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB178" t="n">
         <v>0</v>
       </c>
       <c r="AC178" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.118535+00:00</t>
+          <t>2026-10-27T15:50:17.571639+00:00</t>
         </is>
       </c>
       <c r="AD178" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "fnguide_consensus", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE178" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF178" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG178" t="inlineStr">
@@ -26377,7 +26537,7 @@
       <c r="S180" t="inlineStr"/>
       <c r="T180" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U180" t="inlineStr">
@@ -26392,7 +26552,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X180" t="inlineStr">
@@ -26409,29 +26569,29 @@
         <v>1</v>
       </c>
       <c r="AA180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB180" t="n">
         <v>0</v>
       </c>
       <c r="AC180" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.314362+00:00</t>
+          <t>2026-10-27T15:50:18.934585+00:00</t>
         </is>
       </c>
       <c r="AD180" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "google_trends", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE180" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF180" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG180" t="inlineStr">
@@ -26508,7 +26668,7 @@
       <c r="S181" t="inlineStr"/>
       <c r="T181" t="inlineStr">
         <is>
-          <t>미확보(미시도)</t>
+          <t>미확보(시도 실패)</t>
         </is>
       </c>
       <c r="U181" t="inlineStr">
@@ -26523,7 +26683,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>Individual source access and collection not executed in this run</t>
+          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
         </is>
       </c>
       <c r="X181" t="inlineStr">
@@ -26540,29 +26700,29 @@
         <v>1</v>
       </c>
       <c r="AA181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB181" t="n">
         <v>0</v>
       </c>
       <c r="AC181" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.353566+00:00</t>
+          <t>2026-10-27T15:50:21.035894+00:00</t>
         </is>
       </c>
       <c r="AD181" t="inlineStr">
         <is>
-          <t>{"local": null, "db": null, "fred": "NO_VERIFIED_FRED_MAPPING"}</t>
+          <t>{"shared_probe_group": "reddit_api", "http_status": 200, "result": "DOWNLOADED_SOURCE_PAGE_NOT_INDICATOR_SERIES"}</t>
         </is>
       </c>
       <c r="AE181" t="inlineStr">
         <is>
-          <t>No implemented official data adapter or local source for this indicator</t>
+          <t>Source-access result only; no verified historical indicator observations</t>
         </is>
       </c>
       <c r="AF181" t="inlineStr">
         <is>
-          <t>Identify a licensed official data endpoint and independent fallback</t>
+          <t>Find licensed historical observations or independent provider with dated releases</t>
         </is>
       </c>
       <c r="AG181" t="inlineStr">

</xml_diff>

<commit_message>
Audit all 190 indicators and derive Korean rate components
</commit_message>
<xml_diff>
--- a/market-history/research/regime190/inventory_190.xlsx
+++ b/market-history/research/regime190/inventory_190.xlsx
@@ -7428,8 +7428,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -7440,41 +7448,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
@@ -7488,17 +7516,17 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA42" t="n">
         <v>0</v>
       </c>
       <c r="AB42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC42" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.004638+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD42" t="inlineStr">
@@ -7508,17 +7536,17 @@
       </c>
       <c r="AE42" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH42" t="inlineStr">
@@ -7526,7 +7554,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7559,8 +7591,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -7571,41 +7611,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4547508</t>
         </is>
       </c>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
@@ -7619,17 +7679,17 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA43" t="n">
         <v>0</v>
       </c>
       <c r="AB43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.008673+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD43" t="inlineStr">
@@ -7639,17 +7699,17 @@
       </c>
       <c r="AE43" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH43" t="inlineStr">
@@ -7657,7 +7717,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7690,8 +7754,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -7702,41 +7774,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4535546</t>
         </is>
       </c>
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -7750,17 +7842,17 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA44" t="n">
         <v>0</v>
       </c>
       <c r="AB44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.014227+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD44" t="inlineStr">
@@ -7770,17 +7862,17 @@
       </c>
       <c r="AE44" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH44" t="inlineStr">
@@ -7788,7 +7880,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7821,8 +7917,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -7833,41 +7937,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
@@ -7881,17 +8005,17 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA45" t="n">
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC45" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.021551+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD45" t="inlineStr">
@@ -7901,17 +8025,17 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH45" t="inlineStr">
@@ -7919,7 +8043,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7952,8 +8080,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -7964,41 +8100,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
@@ -8012,17 +8168,17 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA46" t="n">
         <v>0</v>
       </c>
       <c r="AB46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC46" t="inlineStr">
         <is>
-          <t>2026-10-27T15:31:12.260327+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD46" t="inlineStr">
@@ -8032,17 +8188,17 @@
       </c>
       <c r="AE46" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH46" t="inlineStr">
@@ -8050,7 +8206,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8083,8 +8243,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -8095,41 +8263,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4549899</t>
         </is>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
@@ -8143,17 +8331,17 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA47" t="n">
         <v>0</v>
       </c>
       <c r="AB47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC47" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.032750+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD47" t="inlineStr">
@@ -8163,17 +8351,17 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH47" t="inlineStr">
@@ -8181,7 +8369,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8476,8 +8668,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -8488,41 +8688,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4535512</t>
         </is>
       </c>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
@@ -8536,17 +8756,17 @@
         </is>
       </c>
       <c r="Z50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA50" t="n">
         <v>0</v>
       </c>
       <c r="AB50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.046349+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr">
@@ -8556,17 +8776,17 @@
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH50" t="inlineStr">
@@ -8574,7 +8794,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8738,8 +8962,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>read-only KIS daily OHLCV per-symbol derivation</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -8750,41 +8982,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>see private per-symbol manifest</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>daily_per_symbol</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2011-09-16</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4605978</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4547612</t>
         </is>
       </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>DERIVED_MARKET_MAPPING_UNVERIFIED</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Actual per-symbol series exists; 2011-2026 historical market membership and PIT timestamps are unverified</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
@@ -8798,17 +9050,17 @@
         </is>
       </c>
       <c r="Z52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA52" t="n">
         <v>0</v>
       </c>
       <c r="AB52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC52" t="inlineStr">
         <is>
-          <t>2026-10-27T15:29:06.502256+00:00</t>
+          <t>2026-10-29T14:20:14.947107+00:00</t>
         </is>
       </c>
       <c r="AD52" t="inlineStr">
@@ -8818,17 +9070,17 @@
       </c>
       <c r="AE52" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>Actual per-symbol OHLCV derived; historical market identity and PIT remain unverified</t>
         </is>
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Verify as-of market membership, KIS adjustments, exact formula and release time</t>
         </is>
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH52" t="inlineStr">
@@ -8836,7 +9088,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>private:db_daily_price_derived/*.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -16242,8 +16498,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>read-only Korean market rate DB series</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -16254,41 +16518,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
-      <c r="N108" t="inlineStr"/>
-      <c r="O108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>64f465235dba19acaea6a3aa5fd89862b39882ac378a2c4ae973d7c053edf2c2</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>daily_rate</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="R108" t="inlineStr"/>
       <c r="S108" t="inlineStr"/>
       <c r="T108" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U108" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V108" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL_HISTORY_PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="W108" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Only 2025-2026; 109 lacks MSB, 110 lacks BBB, and release vintages are unverified</t>
         </is>
       </c>
       <c r="X108" t="inlineStr">
@@ -16302,17 +16586,17 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA108" t="n">
         <v>0</v>
       </c>
       <c r="AB108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC108" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:45.087750+00:00</t>
+          <t>2026-10-29T14:20:51.642809+00:00</t>
         </is>
       </c>
       <c r="AD108" t="inlineStr">
@@ -16322,17 +16606,17 @@
       </c>
       <c r="AE108" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>2025-2026 rate series derived; missing subcomponents, full history and PIT vintages</t>
         </is>
       </c>
       <c r="AF108" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Acquire earlier official history and release vintages; verify missing MSB and BBB series</t>
         </is>
       </c>
       <c r="AG108" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH108" t="inlineStr">
@@ -16340,7 +16624,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI108" t="inlineStr"/>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -16373,8 +16661,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>read-only Korean market rate DB series</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I109" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -16385,41 +16681,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
-      <c r="N109" t="inlineStr"/>
-      <c r="O109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>64f465235dba19acaea6a3aa5fd89862b39882ac378a2c4ae973d7c053edf2c2</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>daily_rate</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="R109" t="inlineStr"/>
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL_HISTORY_PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Only 2025-2026; 109 lacks MSB, 110 lacks BBB, and release vintages are unverified</t>
         </is>
       </c>
       <c r="X109" t="inlineStr">
@@ -16433,17 +16749,17 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA109" t="n">
         <v>0</v>
       </c>
       <c r="AB109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC109" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:59.182768+00:00</t>
+          <t>2026-10-29T14:20:51.642809+00:00</t>
         </is>
       </c>
       <c r="AD109" t="inlineStr">
@@ -16453,17 +16769,17 @@
       </c>
       <c r="AE109" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>2025-2026 rate series derived; missing subcomponents, full history and PIT vintages</t>
         </is>
       </c>
       <c r="AF109" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Acquire earlier official history and release vintages; verify missing MSB and BBB series</t>
         </is>
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH109" t="inlineStr">
@@ -16471,7 +16787,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI109" t="inlineStr"/>
+      <c r="AI109" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -16504,8 +16824,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>read-only Korean market rate DB series</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -16516,41 +16844,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
-      <c r="M110" t="inlineStr"/>
-      <c r="N110" t="inlineStr"/>
-      <c r="O110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>64f465235dba19acaea6a3aa5fd89862b39882ac378a2c4ae973d7c053edf2c2</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>daily_rate</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="R110" t="inlineStr"/>
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V110" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL_HISTORY_PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Only 2025-2026; 109 lacks MSB, 110 lacks BBB, and release vintages are unverified</t>
         </is>
       </c>
       <c r="X110" t="inlineStr">
@@ -16564,17 +16912,17 @@
         </is>
       </c>
       <c r="Z110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA110" t="n">
         <v>0</v>
       </c>
       <c r="AB110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC110" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:45.141452+00:00</t>
+          <t>2026-10-29T14:20:51.642809+00:00</t>
         </is>
       </c>
       <c r="AD110" t="inlineStr">
@@ -16584,17 +16932,17 @@
       </c>
       <c r="AE110" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>2025-2026 rate series derived; missing subcomponents, full history and PIT vintages</t>
         </is>
       </c>
       <c r="AF110" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Acquire earlier official history and release vintages; verify missing MSB and BBB series</t>
         </is>
       </c>
       <c r="AG110" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH110" t="inlineStr">
@@ -16602,7 +16950,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI110" t="inlineStr"/>
+      <c r="AI110" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -16635,8 +16987,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>read-only Korean market rate DB series</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -16647,41 +17007,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
-      <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>64f465235dba19acaea6a3aa5fd89862b39882ac378a2c4ae973d7c053edf2c2</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>daily_rate</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="R111" t="inlineStr"/>
       <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL_HISTORY_PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Only 2025-2026; 109 lacks MSB, 110 lacks BBB, and release vintages are unverified</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">
@@ -16695,17 +17075,17 @@
         </is>
       </c>
       <c r="Z111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA111" t="n">
         <v>0</v>
       </c>
       <c r="AB111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC111" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:45.144242+00:00</t>
+          <t>2026-10-29T14:20:51.642809+00:00</t>
         </is>
       </c>
       <c r="AD111" t="inlineStr">
@@ -16715,17 +17095,17 @@
       </c>
       <c r="AE111" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>2025-2026 rate series derived; missing subcomponents, full history and PIT vintages</t>
         </is>
       </c>
       <c r="AF111" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Acquire earlier official history and release vintages; verify missing MSB and BBB series</t>
         </is>
       </c>
       <c r="AG111" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH111" t="inlineStr">
@@ -16733,7 +17113,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI111" t="inlineStr"/>
+      <c r="AI111" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -16766,8 +17150,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>read-only Korean market rate DB series</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>private read-only PostgreSQL source</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr">
         <is>
           <t>unreviewed</t>
@@ -16778,41 +17170,61 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>64f465235dba19acaea6a3aa5fd89862b39882ac378a2c4ae973d7c053edf2c2</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>daily_rate</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>325</t>
         </is>
       </c>
       <c r="R112" t="inlineStr"/>
       <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr">
         <is>
-          <t>미확보(시도 실패)</t>
+          <t>일부 확보</t>
         </is>
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
+          <t>PARTIAL_HISTORY_PIT_UNVERIFIED</t>
         </is>
       </c>
       <c r="W112" t="inlineStr">
         <is>
-          <t>Candidate source was queried but the indicator-specific required fields, scope, or rights were not verified</t>
+          <t>Only 2025-2026; 109 lacks MSB, 110 lacks BBB, and release vintages are unverified</t>
         </is>
       </c>
       <c r="X112" t="inlineStr">
@@ -16826,17 +17238,17 @@
         </is>
       </c>
       <c r="Z112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA112" t="n">
         <v>0</v>
       </c>
       <c r="AB112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC112" t="inlineStr">
         <is>
-          <t>2026-10-27T15:30:45.148907+00:00</t>
+          <t>2026-10-29T14:20:51.642809+00:00</t>
         </is>
       </c>
       <c r="AD112" t="inlineStr">
@@ -16846,17 +17258,17 @@
       </c>
       <c r="AE112" t="inlineStr">
         <is>
-          <t>DB field candidate observed but indicator-specific mapping unverified</t>
+          <t>2025-2026 rate series derived; missing subcomponents, full history and PIT vintages</t>
         </is>
       </c>
       <c r="AF112" t="inlineStr">
         <is>
-          <t>Validate field, instrument universe, dates, and market</t>
+          <t>Acquire earlier official history and release vintages; verify missing MSB and BBB series</t>
         </is>
       </c>
       <c r="AG112" t="inlineStr">
         <is>
-          <t>NEEDS_REVIEW</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="AH112" t="inlineStr">
@@ -16864,7 +17276,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="AI112" t="inlineStr"/>
+      <c r="AI112" t="inlineStr">
+        <is>
+          <t>private:db_rates_derived.csv.gz</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">

</xml_diff>